<commit_message>
Added all unit scripts. halfway point in testing. added all factions. did some research into historical commanders. started to align work with the ability to select allies.
</commit_message>
<xml_diff>
--- a/assets/ESR Command Generic-Austrian Commanders.xlsx
+++ b/assets/ESR Command Generic-Austrian Commanders.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9efa18f7c2e81ea4/Documents/NewRecruit/ESR_NewRecruit/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9EFA18F7C2E81EA4/Documents/NewRecruit/ESR_NewRecruit/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{BE457ED5-2306-4118-913C-FC17988DB954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5CEE133-8DA0-412A-90AA-A0659D20FD15}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="8_{BE457ED5-2306-4118-913C-FC17988DB954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DB8B7A9-410F-4361-81B4-61FDF0393DBB}"/>
   <bookViews>
-    <workbookView xWindow="10110" yWindow="765" windowWidth="18525" windowHeight="14115" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3390" yWindow="210" windowWidth="26610" windowHeight="14595" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <r>
       <rPr>
@@ -108,25 +108,37 @@
     <t>Avantgarde Division</t>
   </si>
   <si>
-    <t>Generalleutenant</t>
-  </si>
-  <si>
     <t>Infanterie Division</t>
   </si>
   <si>
     <t>Reservieren Division</t>
   </si>
   <si>
-    <t>Generalmajor</t>
-  </si>
-  <si>
     <t>Kavallerie Brigade</t>
   </si>
   <si>
     <t>Korps Reservieren</t>
   </si>
   <si>
-    <t>Geralleutenant</t>
+    <t>AU Geralleutenant Avantgarde</t>
+  </si>
+  <si>
+    <t>AU Generalleutenant Infantrie</t>
+  </si>
+  <si>
+    <t>AU Generalleutenant Reservieren</t>
+  </si>
+  <si>
+    <t>AU Generalmajor Kavallerie</t>
+  </si>
+  <si>
+    <t>AU Generalmajor Reservieren</t>
+  </si>
+  <si>
+    <t>Nation</t>
+  </si>
+  <si>
+    <t>Austria</t>
   </si>
 </sst>
 </file>
@@ -303,9 +315,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -314,18 +338,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -635,214 +647,232 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="14" style="5" customWidth="1"/>
-    <col min="3" max="4" width="10.5" customWidth="1"/>
-    <col min="5" max="5" width="11.5" customWidth="1"/>
-    <col min="6" max="6" width="10.5" customWidth="1"/>
-    <col min="7" max="7" width="12.33203125" customWidth="1"/>
-    <col min="8" max="8" width="26" customWidth="1"/>
-    <col min="9" max="9" width="9.33203125" customWidth="1"/>
-    <col min="10" max="10" width="10.5" customWidth="1"/>
-    <col min="11" max="11" width="62.83203125" customWidth="1"/>
-    <col min="12" max="12" width="8" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="14" style="5" customWidth="1"/>
+    <col min="4" max="5" width="10.5" customWidth="1"/>
+    <col min="6" max="6" width="11.5" customWidth="1"/>
+    <col min="7" max="7" width="10.5" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
+    <col min="10" max="10" width="9.33203125" customWidth="1"/>
+    <col min="11" max="11" width="10.5" customWidth="1"/>
+    <col min="12" max="12" width="62.83203125" customWidth="1"/>
+    <col min="13" max="13" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="63.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="6"/>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
+    <row r="1" spans="1:13" ht="63.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
     </row>
-    <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="10" t="s">
+    <row r="2" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="C2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="9"/>
-      <c r="F2" s="1" t="s">
+      <c r="E2" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="13"/>
+      <c r="G2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
     </row>
-    <row r="3" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="7"/>
-      <c r="B3" s="3"/>
+    <row r="3" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="11"/>
       <c r="C3" s="3"/>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3"/>
+      <c r="E3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
-      <c r="I3" s="2"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="12" t="s">
+    <row r="4" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="8">
+        <v>1</v>
+      </c>
+      <c r="E4" s="8">
+        <v>0</v>
+      </c>
+      <c r="F4" s="8">
+        <v>0</v>
+      </c>
+      <c r="G4" s="8">
+        <v>1</v>
+      </c>
+      <c r="H4" s="8">
+        <v>1</v>
+      </c>
+      <c r="I4" s="7"/>
+      <c r="J4" s="5"/>
+    </row>
+    <row r="5" spans="1:13" ht="51.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="8">
+        <v>1</v>
+      </c>
+      <c r="E5" s="8">
+        <v>0</v>
+      </c>
+      <c r="F5" s="8">
+        <v>0</v>
+      </c>
+      <c r="G5" s="8">
+        <v>1</v>
+      </c>
+      <c r="H5" s="8">
+        <v>1</v>
+      </c>
+      <c r="I5" s="7"/>
+      <c r="J5" s="5"/>
+    </row>
+    <row r="6" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="13">
-        <v>1</v>
-      </c>
-      <c r="D4" s="13">
+      <c r="C6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="8">
+        <v>1</v>
+      </c>
+      <c r="E6" s="8">
         <v>0</v>
       </c>
-      <c r="E4" s="13">
+      <c r="F6" s="8">
         <v>0</v>
       </c>
-      <c r="F4" s="13">
-        <v>1</v>
-      </c>
-      <c r="G4" s="13">
-        <v>1</v>
-      </c>
-      <c r="H4" s="12"/>
-      <c r="I4" s="5"/>
+      <c r="G6" s="8">
+        <v>1</v>
+      </c>
+      <c r="H6" s="8">
+        <v>1</v>
+      </c>
+      <c r="I6" s="7"/>
+      <c r="J6" s="2"/>
     </row>
-    <row r="5" spans="1:12" ht="51.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="13">
-        <v>1</v>
-      </c>
-      <c r="D5" s="13">
+    <row r="7" spans="1:13" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="8">
+        <v>1</v>
+      </c>
+      <c r="E7" s="8">
         <v>0</v>
       </c>
-      <c r="E5" s="13">
+      <c r="F7" s="8">
         <v>0</v>
       </c>
-      <c r="F5" s="13">
-        <v>1</v>
-      </c>
-      <c r="G5" s="13">
-        <v>1</v>
-      </c>
-      <c r="H5" s="12"/>
-      <c r="I5" s="5"/>
+      <c r="G7" s="8">
+        <v>1</v>
+      </c>
+      <c r="H7" s="8">
+        <v>1</v>
+      </c>
+      <c r="I7" s="7"/>
     </row>
-    <row r="6" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="13">
-        <v>1</v>
-      </c>
-      <c r="D6" s="13">
-        <v>0</v>
-      </c>
-      <c r="E6" s="13">
-        <v>0</v>
-      </c>
-      <c r="F6" s="13">
-        <v>1</v>
-      </c>
-      <c r="G6" s="13">
-        <v>1</v>
-      </c>
-      <c r="H6" s="12"/>
-      <c r="I6" s="2"/>
+    <row r="8" spans="1:13" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="8">
+        <v>1</v>
+      </c>
+      <c r="E8" s="8">
+        <v>1</v>
+      </c>
+      <c r="F8" s="8">
+        <v>1</v>
+      </c>
+      <c r="G8" s="8">
+        <v>1</v>
+      </c>
+      <c r="H8" s="8">
+        <v>1</v>
+      </c>
+      <c r="I8" s="7"/>
     </row>
-    <row r="7" spans="1:12" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A7" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="13">
-        <v>1</v>
-      </c>
-      <c r="D7" s="13">
-        <v>0</v>
-      </c>
-      <c r="E7" s="13">
-        <v>0</v>
-      </c>
-      <c r="F7" s="13">
-        <v>1</v>
-      </c>
-      <c r="G7" s="13">
-        <v>1</v>
-      </c>
-      <c r="H7" s="12"/>
-    </row>
-    <row r="8" spans="1:12" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A8" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="13">
-        <v>1</v>
-      </c>
-      <c r="D8" s="13">
-        <v>1</v>
-      </c>
-      <c r="E8" s="13">
-        <v>1</v>
-      </c>
-      <c r="F8" s="13">
-        <v>1</v>
-      </c>
-      <c r="G8" s="13">
-        <v>1</v>
-      </c>
-      <c r="H8" s="12"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="12"/>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="B1:M1"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="E2:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>